<commit_message>
refactor: finish migration cleanup — fix imports, upgrade semantic search, relocate tests
- Fix tracing.py import (import config → from tamubot.core import config)
- Upgrade semantic_search to hybrid (vector + BM25 via RRF)
- Move 3 test files from src/ to tests/
- Remove stale superpowers plan/spec docs
- Normalize line endings and formatting
- Update golden set, add test_hooks.sh to .gitignore

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tamu_data/evals/golden_sets/CSCE_25gradcourses_nonrecursive.xlsx
+++ b/tamu_data/evals/golden_sets/CSCE_25gradcourses_nonrecursive.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,16 @@
           <t>run:CSCE_25gradcourses_20260418_20260418_090845</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>run:cs250_ov50_20260425_214025</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>run:cs250_ov50_ragas_20260426_002345</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="86.40000000000001" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -568,6 +578,16 @@
           <t>CSCE 611 §? 0.68, CSCE 611 §? 0.54</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.71, CSCE 611 §? 0.70, CSCE 611 §? 0.62, CSCE 611 §? 0.59, CSCE 611 §? 0.57, CSCE 611 §? 0.52</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.71, CSCE 611 §? 0.70, CSCE 611 §? 0.62, CSCE 611 §? 0.59, CSCE 611 §? 0.57, CSCE 611 §? 0.52</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="172.8" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -617,6 +637,16 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>CSCE 612 §? 0.89, CSCE 612 §? 0.65</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>CSCE 612 §? 0.86, CSCE 612 §? 0.84</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>CSCE 612 §? 0.86, CSCE 612 §? 0.84</t>
         </is>
       </c>
     </row>
@@ -671,6 +701,16 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>CSCE 669 §? 0.80, CSCE 669 §? 0.51</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>CSCE 669 §? 0.71, CSCE 669 §? 0.70</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>CSCE 669 §? 0.71, CSCE 669 §? 0.70</t>
         </is>
       </c>
     </row>
@@ -726,6 +766,16 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>CSCE 665 §? 0.93, CSCE 665 §? 0.79</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.93, CSCE 665 §? 0.81</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.93, CSCE 665 §? 0.81</t>
         </is>
       </c>
     </row>
@@ -785,6 +835,16 @@
           <t>CSCE 670 §? 0.89, CSCE 670 §? 0.62</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CSCE 670 §? 0.82, CSCE 670 §? 0.67</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>CSCE 670 §? 0.82, CSCE 670 §? 0.67</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="144" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -836,6 +896,16 @@
           <t>CSCE 676 §? 0.90, CSCE 676 §? 0.60</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>CSCE 676 §? 0.86, CSCE 676 §? 0.55</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>CSCE 676 §? 0.86, CSCE 676 §? 0.55</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="273.6" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -888,6 +958,16 @@
           <t>CSCE 672 §? 0.82, CSCE 672 §? 0.62</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>CSCE 672 §? 0.76, CSCE 672 §? 0.67</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>CSCE 672 §? 0.76, CSCE 672 §? 0.67</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="172.8" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -937,6 +1017,16 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>CSCE 608 §? 0.89, CSCE 608 §? 0.62</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.87, CSCE 608 §? 0.66</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.87, CSCE 608 §? 0.66</t>
         </is>
       </c>
     </row>
@@ -995,6 +1085,16 @@
           <t>CSCE 624 §? 0.84, CSCE 624 §? 0.74</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>CSCE 624 §? 0.70, CSCE 624 §? 0.70, CSCE 624 §? 0.70</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>CSCE 624 §? 0.70, CSCE 624 §? 0.70, CSCE 624 §? 0.70</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="216" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -1048,6 +1148,16 @@
           <t>CSCE 629 §? 0.85, CSCE 629 §? 0.52</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>CSCE 629 §? 0.88, CSCE 629 §? 0.60</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CSCE 629 §? 0.88, CSCE 629 §? 0.60</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="158.4" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -1097,6 +1207,16 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>CSCE 638 §? 0.58, CSCE 638 §? 0.55</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>CSCE 638 §? 0.67, CSCE 638 §? 0.62</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>CSCE 638 §? 0.67, CSCE 638 §? 0.62</t>
         </is>
       </c>
     </row>
@@ -1162,6 +1282,16 @@
           <t>CSCE 656 §? 0.80, CSCE 656 §? 0.59</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>CSCE 656 §? 0.61, CSCE 656 §? 0.52, CSCE 656 §? 0.52</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>CSCE 656 §? 0.61, CSCE 656 §? 0.52, CSCE 656 §? 0.52</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="201.6" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -1212,6 +1342,16 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>CSCE 665 §? 0.75, CSCE 665 §? 0.54</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.69, CSCE 665 §? 0.55, CSCE 665 §? 0.55</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.69, CSCE 665 §? 0.55, CSCE 665 §? 0.55</t>
         </is>
       </c>
     </row>
@@ -1270,6 +1410,16 @@
           <t>CSCE 641 §? 0.79, CSCE 641 §? 0.61</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>CSCE 641 §? 0.79, CSCE 641 §? 0.78</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>CSCE 641 §? 0.79, CSCE 641 §? 0.78</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="302.4" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -1325,6 +1475,16 @@
           <t>CSCE 672 §? 0.80, CSCE 672 §? 0.68</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>CSCE 672 §? 0.75, CSCE 672 §? 0.71</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>CSCE 672 §? 0.75, CSCE 672 §? 0.71</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="187.2" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1380,6 +1540,16 @@
           <t>CSCE 608 §? 0.66, CSCE 608 §? 0.47</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.67, CSCE 608 §? 0.63</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.67, CSCE 608 §? 0.63</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="158.4" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1430,6 +1600,16 @@
           <t>CSCE 605 §? 0.68, CSCE 681 §? 0.63, CSCE 713 §? 0.63, CSCE 629 §? 0.62, CSCE 681 §? 0.59, CSCE 652 §? 0.59, CSCE 614 §? 0.59, ISEN 620 §? 0.59, CSCE 635 §? 0.57, ISEN 620 §? 0.57</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>CSCE 681 §? 0.62, CSCE 681 §? 0.61, CSCE 681 §? 0.61, CSCE 681 §? 0.60, CSCE 632 §? 0.60, CSCE 629 §? 0.57, ISEN 441 §? 0.57, CSCE 624 §? 0.55, CSCE 111 §? 0.54, CSCE 111 §? 0.54</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>CSCE 681 §? 0.62, CSCE 681 §? 0.61, CSCE 681 §? 0.61, CSCE 681 §? 0.60, CSCE 632 §? 0.60, CSCE 629 §? 0.57, ISEN 441 §? 0.57, CSCE 624 §? 0.55, CSCE 111 §? 0.54, CSCE 111 §? 0.54</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="86.40000000000001" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -1480,6 +1660,16 @@
           <t>CSCE 672 §? 0.75, CSCE 672 §? 0.52</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>CSCE 672 §? 0.75, CSCE 672 §? 0.75, CSCE 672 §? 0.73, CSCE 672 §? 0.70</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>CSCE 672 §? 0.75, CSCE 672 §? 0.75, CSCE 672 §? 0.73, CSCE 672 §? 0.70</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="86.40000000000001" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1530,6 +1720,16 @@
           <t>CSCE 652 §? 0.55, CSCE 652 §? 0.50, CSCE 605 §? 0.47, CSCE 605 §? 0.46, CSCE 676 §? 0.45, CSCE 632 §? 0.44, ISEN 620 §? 0.44, ISEN 620 §? 0.43, CSCE 713 §? 0.43, CSCE 633 §? 0.41</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>CSCE 629 §? 0.61, CSCE 629 §? 0.59, ISEN 441 §? 0.58, CSCE 629 §? 0.58, CSCE 652 §? 0.56</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>CSCE 629 §? 0.61, CSCE 629 §? 0.59, ISEN 441 §? 0.58, CSCE 629 §? 0.58, CSCE 652 §? 0.56</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="100.8" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1580,6 +1780,16 @@
           <t>CSCE 638 §? 0.72, CSCE 670 §? 0.61</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>CSCE 638 §? 0.71, CSCE 638 §? 0.71, CSCE 638 §? 0.70, CSCE 670 §? 0.70, CSCE 638 §? 0.68, CSCE 638 §? 0.68</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>CSCE 638 §? 0.71, CSCE 638 §? 0.71, CSCE 638 §? 0.70, CSCE 670 §? 0.70, CSCE 638 §? 0.68, CSCE 638 §? 0.68</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="129.6" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1630,6 +1840,16 @@
           <t>CSCE 681 §? 0.77, CSCE 672 §? 0.51</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>CSCE 681 §? 0.75, CSCE 681 §? 0.69</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>CSCE 681 §? 0.75, CSCE 681 §? 0.69</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="144" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -1680,6 +1900,16 @@
           <t>ISEN 620 §? 0.49, CSCE 614 §? 0.48, CSCE 681 §? 0.47, CSCE 633 §? 0.46, CSCE 681 §? 0.44, CSCE 605 §? 0.43, CSCE 608 §? 0.43, CSCE 605 §? 0.41, ISEN 620 §? 0.41, CSCE 605 §? 0.40</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>CSCE 635 §? 0.57, CSCE 656 §? 0.55, CSCE 421 §? 0.54, CSCE 633 §? 0.52, CSCE 633 §? 0.52, CSCE 672 §? 0.51, CSCE 672 §? 0.51, CSCE 672 §? 0.51, CSCE 672 §? 0.50, CSCE 633 §? 0.50</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>CSCE 635 §? 0.57, CSCE 656 §? 0.55, CSCE 421 §? 0.54, CSCE 633 §? 0.52, CSCE 633 §? 0.52, CSCE 672 §? 0.51, CSCE 672 §? 0.51, CSCE 672 §? 0.51, CSCE 672 §? 0.50, CSCE 633 §? 0.50</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="86.40000000000001" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -1730,6 +1960,16 @@
           <t>CSCE 679 §? 0.81, CSCE 679 §? 0.55</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>CSCE 679 §? 0.81, CSCE 679 §? 0.81, CSCE 679 §? 0.80, CSCE 679 §? 0.77</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>CSCE 679 §? 0.81, CSCE 679 §? 0.81, CSCE 679 §? 0.80, CSCE 679 §? 0.77</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28.8" customHeight="1">
       <c r="A25" s="2" t="n">
@@ -1778,6 +2018,16 @@
       <c r="L25" t="inlineStr">
         <is>
           <t>CSCE 629 §? 0.74, CSCE 629 §? 0.70</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>CSCE 629 §? 0.78, CSCE 629 §? 0.70, CSCE 629 §? 0.57, CSCE 629 §? 0.55</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CSCE 629 §? 0.78, CSCE 629 §? 0.70, CSCE 629 §? 0.57, CSCE 629 §? 0.55</t>
         </is>
       </c>
     </row>
@@ -1836,6 +2086,16 @@
           <t>CSCE 608 §? 0.88, CSCE 608 §? 0.41</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.73, CSCE 608 §? 0.56</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.73, CSCE 608 §? 0.56</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="43.2" customHeight="1">
       <c r="A27" s="2" t="n">
@@ -1884,6 +2144,16 @@
       <c r="L27" t="inlineStr">
         <is>
           <t>CSCE 633 §? 0.71, CSCE 633 §? 0.47</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>CSCE 633 §? 0.75, CSCE 633 §? 0.47</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>CSCE 633 §? 0.75, CSCE 633 §? 0.47</t>
         </is>
       </c>
     </row>
@@ -1938,6 +2208,16 @@
       <c r="L28" t="inlineStr">
         <is>
           <t>CSCE 633 §? 0.84, CSCE 633 §? 0.57</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>CSCE 633 §? 0.76, CSCE 633 §? 0.60</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>CSCE 633 §? 0.76, CSCE 633 §? 0.60</t>
         </is>
       </c>
     </row>
@@ -1996,6 +2276,16 @@
           <t>CSCE 665 §? 0.85, CSCE 665 §? 0.59</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.80, CSCE 665 §? 0.75</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.80, CSCE 665 §? 0.75</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="144" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -2050,6 +2340,16 @@
           <t>CSCE 669 §? 0.79, CSCE 669 §? 0.48</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>CSCE 669 §? 0.71, CSCE 669 §? 0.66</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CSCE 669 §? 0.71, CSCE 669 §? 0.66</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="144" customHeight="1">
       <c r="A31" s="2" t="n">
@@ -2104,6 +2404,16 @@
           <t>CSCE 665 §? 0.84, CSCE 665 §? 0.70</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.76, CSCE 665 §? 0.71, CSCE 665 §? 0.64</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CSCE 665 §? 0.76, CSCE 665 §? 0.71, CSCE 665 §? 0.64</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="57.6" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -2154,6 +2464,16 @@
           <t>CSCE 608 §? 0.91, CSCE 608 §? 0.64</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.88, CSCE 608 §? 0.70</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CSCE 608 §? 0.88, CSCE 608 §? 0.70</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="72" customHeight="1">
       <c r="A33" s="2" t="n">
@@ -2202,6 +2522,16 @@
       <c r="L33" t="inlineStr">
         <is>
           <t>CSCE 681 §? 0.87, CSCE 681 §? 0.50</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>CSCE 681 §? 0.72, CSCE 681 §? 0.70</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>CSCE 681 §? 0.72, CSCE 681 §? 0.70</t>
         </is>
       </c>
     </row>
@@ -2258,6 +2588,16 @@
           <t>CSCE 611 §? 0.80, CSCE 611 §? 0.76</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.79, CSCE 611 §? 0.74, CSCE 611 §? 0.69, CSCE 611 §? 0.68, CSCE 611 §? 0.68</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>CSCE 611 §? 0.79, CSCE 611 §? 0.74, CSCE 611 §? 0.69, CSCE 611 §? 0.68, CSCE 611 §? 0.68</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="244.8" customHeight="1">
       <c r="A35" s="2" t="n">
@@ -2310,6 +2650,16 @@
       <c r="L35" t="inlineStr">
         <is>
           <t>CSCE 670 §? 0.72, CSCE 670 §? 0.71</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>CSCE 670 §? 0.68, CSCE 670 §? 0.65, CSCE 670 §? 0.59</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>CSCE 670 §? 0.68, CSCE 670 §? 0.65, CSCE 670 §? 0.59</t>
         </is>
       </c>
     </row>
@@ -2368,6 +2718,16 @@
           <t>CSCE 632 §? 0.80, CSCE 632 §? 0.77, CSCE 632 §? 0.73</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>CSCE 632 §? 0.73, CSCE 632 §? 0.71, CSCE 632 §? 0.69, CSCE 632 §? 0.65</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>CSCE 632 §? 0.73, CSCE 632 §? 0.71, CSCE 632 §? 0.69, CSCE 632 §? 0.65</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="201.6" customHeight="1">
       <c r="A37" s="2" t="n">
@@ -2422,6 +2782,16 @@
           <t>CSCE 669 §? 0.85, CSCE 669 §? 0.78</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>CSCE 669 §? 0.78, CSCE 669 §? 0.55</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>CSCE 669 §? 0.78, CSCE 669 §? 0.55</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="259.2" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -2474,6 +2844,16 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>CSCE 670 §? 0.79, CSCE 670 §? 0.46</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>CSCE 670 §? 0.80, CSCE 670 §? 0.56</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>CSCE 670 §? 0.80, CSCE 670 §? 0.56</t>
         </is>
       </c>
     </row>

</xml_diff>